<commit_message>
pdf verson of splitsync wireframe created
</commit_message>
<xml_diff>
--- a/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
+++ b/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amsh/Education/CDU - PRT585 SOFTWARE ENGINEERING PRACTICE/prt585-software-engineering-team-logs/AmshShrestha_S394695/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA0DBAE-4A85-974F-ADAE-4BA2DE06E160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E3532F-91D9-9D4D-917C-7092EC24D47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Individual Timesheets for all s" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="24">
   <si>
     <t>Week</t>
   </si>
@@ -83,6 +83,15 @@
   </si>
   <si>
     <t>Scaffold PWA react and .net monorepos</t>
+  </si>
+  <si>
+    <t>Week 05</t>
+  </si>
+  <si>
+    <t>Update wireframe</t>
+  </si>
+  <si>
+    <t>Design Authentication page</t>
   </si>
 </sst>
 </file>
@@ -104,12 +113,14 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -647,6 +658,89 @@
         <v>5</v>
       </c>
     </row>
+    <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="163" spans="4:4" ht="13" x14ac:dyDescent="0.15">
       <c r="D163" s="3"/>
     </row>

</xml_diff>

<commit_message>
Updated timesheets - week05
</commit_message>
<xml_diff>
--- a/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
+++ b/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amsh/Education/CDU - PRT585 SOFTWARE ENGINEERING PRACTICE/prt585-software-engineering-team-logs/AmshShrestha_S394695/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amsh/Education/CDU - PRT585 SOFTWARE ENGINEERING PRACTICE/splitsync/AmshShrestha_S394695/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20E3532F-91D9-9D4D-917C-7092EC24D47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_3FD934CFD02B77158A4D67C80CAA0D9277159BC2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Individual Timesheets for all s" sheetId="1" r:id="rId1"/>
@@ -20,14 +20,20 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="27">
   <si>
     <t>Week</t>
   </si>
   <si>
+    <t>Student ID</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
+    <t>Hours [1- 6]</t>
+  </si>
+  <si>
     <t>Activity details</t>
   </si>
   <si>
@@ -58,15 +64,9 @@
     <t>Finalised the project</t>
   </si>
   <si>
-    <t>Student ID</t>
-  </si>
-  <si>
     <t>Week 04</t>
   </si>
   <si>
-    <t>Hours [1- 6]</t>
-  </si>
-  <si>
     <t>Updated trello about tasks to perform in week 04</t>
   </si>
   <si>
@@ -92,6 +92,15 @@
   </si>
   <si>
     <t>Design Authentication page</t>
+  </si>
+  <si>
+    <t>Built authentication backend: ASP.NET Core Identity, JWT issuance, register/login by email or username, EF Core + SQLite migration</t>
+  </si>
+  <si>
+    <t>Built homepage and profile pages in React frontend</t>
+  </si>
+  <si>
+    <t>Resolved git rebase conflict merging authentication work with teammates' changes; verified build and tests passed</t>
   </si>
 </sst>
 </file>
@@ -101,7 +110,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m\-d"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -141,12 +150,6 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -413,129 +416,129 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2">
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3" s="2">
         <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2">
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D6" s="2">
         <v>0.5</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="2">
         <v>0.5</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D8" s="2">
         <v>0</v>
@@ -547,13 +550,13 @@
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" s="6">
         <v>0.5</v>
@@ -564,13 +567,13 @@
     </row>
     <row r="11" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D11" s="6">
         <v>1</v>
@@ -581,13 +584,13 @@
     </row>
     <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D12" s="6">
         <v>1</v>
@@ -598,13 +601,13 @@
     </row>
     <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D13" s="6">
         <v>1</v>
@@ -615,13 +618,13 @@
     </row>
     <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14" s="6">
         <v>0.5</v>
@@ -632,13 +635,13 @@
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" s="6">
         <v>0.5</v>
@@ -649,13 +652,13 @@
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -663,10 +666,10 @@
         <v>21</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>22</v>
@@ -677,10 +680,10 @@
         <v>21</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>23</v>
@@ -691,10 +694,16 @@
         <v>21</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D20">
+        <v>3</v>
+      </c>
+      <c r="E20" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -702,10 +711,16 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D21">
+        <v>1.5</v>
+      </c>
+      <c r="E21" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -713,10 +728,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="D22">
+        <v>1.5</v>
+      </c>
+      <c r="E22" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -724,10 +745,10 @@
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -735,17 +756,16 @@
         <v>21</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="163" spans="4:4" ht="13" x14ac:dyDescent="0.15">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="163" spans="4:4" ht="13" customHeight="1" x14ac:dyDescent="0.15">
       <c r="D163" s="3"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Amsh Shrestha timesheets
</commit_message>
<xml_diff>
--- a/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
+++ b/AmshShrestha_S394695/Individual Timesheets - Amsh Shrestha(S394695).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amsh/Education/CDU - PRT585 SOFTWARE ENGINEERING PRACTICE/splitsync/AmshShrestha_S394695/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3FD934CFD02B77158A4D67C80CAA0D9277159BC2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69705904-B1DB-7B4A-82CF-BF9C1498269B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="25">
   <si>
     <t>Week</t>
   </si>
@@ -86,12 +86,6 @@
   </si>
   <si>
     <t>Week 05</t>
-  </si>
-  <si>
-    <t>Update wireframe</t>
-  </si>
-  <si>
-    <t>Design Authentication page</t>
   </si>
   <si>
     <t>Built authentication backend: ASP.NET Core Identity, JWT issuance, register/login by email or username, EF Core + SQLite migration</t>
@@ -401,7 +395,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E163"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="25.1640625" customWidth="1"/>
@@ -671,7 +665,10 @@
       <c r="C18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="D18">
+        <v>3</v>
+      </c>
+      <c r="E18" t="s">
         <v>22</v>
       </c>
     </row>
@@ -685,7 +682,10 @@
       <c r="C19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="D19">
+        <v>1.5</v>
+      </c>
+      <c r="E19" t="s">
         <v>23</v>
       </c>
     </row>
@@ -700,70 +700,14 @@
         <v>7</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E20" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A21" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>1.5</v>
-      </c>
-      <c r="E21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D22">
-        <v>1.5</v>
-      </c>
-      <c r="E22" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A23" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="163" spans="4:4" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="D163" s="3"/>
+    <row r="159" spans="4:4" ht="13" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="D159" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>